<commit_message>
Added reading of non-usual excels (Excels with more data than the table or with the table displaced)
</commit_message>
<xml_diff>
--- a/datos/invalido.xlsx
+++ b/datos/invalido.xlsx
@@ -435,1102 +435,1102 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.2943523700252064</v>
+        <v>0.3642610991371413</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5157560825744407</v>
+        <v>0.4393585701914053</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3590077806327087</v>
+        <v>0.8622101811175628</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.6010142919656931</v>
+        <v>0.4347973968947693</v>
       </c>
       <c r="B3" t="n">
-        <v>0.3083422362884576</v>
+        <v>0.2629513920687184</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1058607099121126</v>
+        <v>0.7144550027917037</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.7508362994412897</v>
+        <v>0.9534742846485205</v>
       </c>
       <c r="B4" t="n">
-        <v>0.7103871989936563</v>
+        <v>0.7478364194288035</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5587692385465212</v>
+        <v>0.5535501018671309</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.6169810928394748</v>
+        <v>0.4869342562026893</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2145210854107733</v>
+        <v>0.3946206049615253</v>
       </c>
       <c r="C5" t="n">
-        <v>0.198397642470565</v>
+        <v>0.8686273284224302</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.7828365745212756</v>
+        <v>0.8459623319139834</v>
       </c>
       <c r="B6" t="n">
-        <v>0.7629205284416021</v>
+        <v>0.7150521764798419</v>
       </c>
       <c r="C6" t="n">
-        <v>0.419381190628348</v>
+        <v>0.9841353262407144</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.7842946063443984</v>
+        <v>0.521491098019836</v>
       </c>
       <c r="B7" t="n">
-        <v>0.242211834800516</v>
+        <v>0.5536828506031738</v>
       </c>
       <c r="C7" t="n">
-        <v>0.4043005981206325</v>
+        <v>0.08590297473869524</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.5722969727703499</v>
+        <v>0.2574839709447263</v>
       </c>
       <c r="B8" t="n">
-        <v>0.448458300752947</v>
+        <v>0.935439306848471</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9085057055727724</v>
+        <v>0.362206318327155</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.6870920992679753</v>
+        <v>0.3109414981373435</v>
       </c>
       <c r="B9" t="n">
-        <v>0.02093816743056054</v>
+        <v>0.3531859871489232</v>
       </c>
       <c r="C9" t="n">
-        <v>0.579144672477646</v>
+        <v>0.590760023730611</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.764498733931839</v>
+        <v>0.9235485709030722</v>
       </c>
       <c r="B10" t="n">
-        <v>0.1634427101394533</v>
+        <v>0.819959338137869</v>
       </c>
       <c r="C10" t="n">
-        <v>0.4515909552885062</v>
+        <v>0.3310786663202981</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.172961771219439</v>
+        <v>0.132501577462024</v>
       </c>
       <c r="B11" t="n">
-        <v>0.8962587872511032</v>
+        <v>0.4361854078553131</v>
       </c>
       <c r="C11" t="n">
-        <v>0.3916037730332497</v>
+        <v>0.6908893957816845</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.9719399720447283</v>
+        <v>0.1579645997602448</v>
       </c>
       <c r="B12" t="n">
-        <v>0.6745307178183558</v>
+        <v>0.6153441821266217</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9310380632395604</v>
+        <v>0.9547386496628771</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.9401215596262095</v>
+        <v>0.8234611284095843</v>
       </c>
       <c r="B13" t="n">
-        <v>0.06991437040796544</v>
+        <v>0.5489742525658842</v>
       </c>
       <c r="C13" t="n">
-        <v>0.402436489596973</v>
+        <v>0.6788943206172632</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.06378216672463344</v>
+        <v>0.4865046164693585</v>
       </c>
       <c r="B14" t="n">
-        <v>0.737205640659318</v>
+        <v>0.6198293260246734</v>
       </c>
       <c r="C14" t="n">
-        <v>0.491212524811426</v>
+        <v>0.3273554218327915</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.926730470129531</v>
+        <v>0.2081017281585414</v>
       </c>
       <c r="B15" t="n">
-        <v>0.8047001976601855</v>
+        <v>0.4742407635052142</v>
       </c>
       <c r="C15" t="n">
-        <v>0.4208823285493358</v>
+        <v>0.7714495235733287</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.9638056566793387</v>
+        <v>0.9469235121667602</v>
       </c>
       <c r="B16" t="n">
-        <v>0.2161752169764937</v>
+        <v>0.9312617306730616</v>
       </c>
       <c r="C16" t="n">
-        <v>0.969994996011484</v>
+        <v>0.9827423910189745</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.8314962202955781</v>
+        <v>0.7461168377830257</v>
       </c>
       <c r="B17" t="n">
-        <v>0.7233343565000334</v>
+        <v>0.1550816135569292</v>
       </c>
       <c r="C17" t="n">
-        <v>0.5070171103565658</v>
+        <v>0.3824229237223835</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.7241716609793941</v>
+        <v>0.913182090289098</v>
       </c>
       <c r="B18" t="n">
-        <v>0.08705483922661628</v>
+        <v>0.7652182636758874</v>
       </c>
       <c r="C18" t="n">
-        <v>0.9873387366349933</v>
+        <v>0.6719487440962053</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.07792306650161718</v>
+        <v>0.4725751022167024</v>
       </c>
       <c r="B19" t="n">
-        <v>0.9241651430922628</v>
+        <v>0.1584509778857712</v>
       </c>
       <c r="C19" t="n">
-        <v>0.8834386676644572</v>
+        <v>0.7813754559820908</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.9328509974939426</v>
+        <v>0.1103366307018246</v>
       </c>
       <c r="B20" t="n">
-        <v>0.4739703088213898</v>
+        <v>0.3394823663165598</v>
       </c>
       <c r="C20" t="n">
-        <v>0.3177213397410099</v>
+        <v>0.4509238652293436</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.04281765587355957</v>
+        <v>0.903295924411914</v>
       </c>
       <c r="B21" t="n">
-        <v>0.9615380065022631</v>
+        <v>0.9752387379495151</v>
       </c>
       <c r="C21" t="n">
-        <v>0.2654505684433529</v>
+        <v>0.18661260434781</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.4012069788035392</v>
+        <v>0.513642651131759</v>
       </c>
       <c r="B22" t="n">
-        <v>0.3730861368971773</v>
+        <v>0.2908779126374178</v>
       </c>
       <c r="C22" t="n">
-        <v>0.4009948297792636</v>
+        <v>0.2416513763615679</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.9561450567152946</v>
+        <v>0.3611804801943612</v>
       </c>
       <c r="B23" t="n">
-        <v>0.1893888749262694</v>
+        <v>0.5605522801558406</v>
       </c>
       <c r="C23" t="n">
-        <v>0.1454389301589601</v>
+        <v>0.1913218371920437</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0.07455615999795118</v>
+        <v>0.9730203588687899</v>
       </c>
       <c r="B24" t="n">
-        <v>0.7843658778782617</v>
+        <v>0.4110373957826468</v>
       </c>
       <c r="C24" t="n">
-        <v>0.1393658773379756</v>
+        <v>0.7555646816097903</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.4177791403068437</v>
+        <v>0.323971971426414</v>
       </c>
       <c r="B25" t="n">
-        <v>0.8491949125374555</v>
+        <v>0.1669673928923394</v>
       </c>
       <c r="C25" t="n">
-        <v>0.3110092695729104</v>
+        <v>0.509330040650285</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.5477315271129407</v>
+        <v>0.2996228984082996</v>
       </c>
       <c r="B26" t="n">
-        <v>0.9244516635236292</v>
+        <v>0.5661809512956646</v>
       </c>
       <c r="C26" t="n">
-        <v>0.5533499752286336</v>
+        <v>0.6833075525779972</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0.2823991820989662</v>
+        <v>0.875993506445928</v>
       </c>
       <c r="B27" t="n">
-        <v>0.7170959825623049</v>
+        <v>0.9558902765282056</v>
       </c>
       <c r="C27" t="n">
-        <v>0.05341588571066136</v>
+        <v>0.4332152602491856</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.4517728781184955</v>
+        <v>0.718793588379087</v>
       </c>
       <c r="B28" t="n">
-        <v>0.06607735112270785</v>
+        <v>0.3547906747599755</v>
       </c>
       <c r="C28" t="n">
-        <v>0.01098362790565066</v>
+        <v>0.5888230144390761</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.5666630005835321</v>
+        <v>0.6485937629614191</v>
       </c>
       <c r="B29" t="n">
-        <v>0.8913425231659072</v>
+        <v>0.195819452171565</v>
       </c>
       <c r="C29" t="n">
-        <v>0.7787267842988881</v>
+        <v>0.4617002665334933</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0.08914518439911889</v>
+        <v>0.3208788751497276</v>
       </c>
       <c r="B30" t="n">
-        <v>0.5545773106605271</v>
+        <v>0.8347857258514697</v>
       </c>
       <c r="C30" t="n">
-        <v>0.3777262756577437</v>
+        <v>0.8261047130838384</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0.2682726931559409</v>
+        <v>0.4486368693960292</v>
       </c>
       <c r="B31" t="n">
-        <v>0.9696197315308822</v>
+        <v>0.6076980897217376</v>
       </c>
       <c r="C31" t="n">
-        <v>0.01406885152122461</v>
+        <v>0.1852126749486049</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0.5488672236689239</v>
+        <v>0.1434360931386645</v>
       </c>
       <c r="B32" t="n">
-        <v>0.4721782078777461</v>
+        <v>0.3310285579544189</v>
       </c>
       <c r="C32" t="n">
-        <v>0.4951866688654909</v>
+        <v>0.6490133912500426</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0.8873979475859194</v>
+        <v>0.8732318620256962</v>
       </c>
       <c r="B33" t="n">
-        <v>0.1137260092298438</v>
+        <v>0.1044027230703831</v>
       </c>
       <c r="C33" t="n">
-        <v>0.3524944223536328</v>
+        <v>0.5947777887979242</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0.8700943472314123</v>
+        <v>0.8993338208758763</v>
       </c>
       <c r="B34" t="n">
-        <v>0.3803037314679061</v>
+        <v>0.1529107547971765</v>
       </c>
       <c r="C34" t="n">
-        <v>0.5271931970188751</v>
+        <v>0.7676449816146649</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.8252264788159835</v>
+        <v>0.9325048043806701</v>
       </c>
       <c r="B35" t="n">
-        <v>0.06004710032146565</v>
+        <v>0.9684686112713446</v>
       </c>
       <c r="C35" t="n">
-        <v>0.03744916620943728</v>
+        <v>0.06020398441737773</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0.07147705441404406</v>
+        <v>0.7917744936645598</v>
       </c>
       <c r="B36" t="n">
-        <v>0.8945825883383831</v>
+        <v>0.3186336153903198</v>
       </c>
       <c r="C36" t="n">
-        <v>0.3349579415495288</v>
+        <v>0.6465507270531345</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0.9607891742350766</v>
+        <v>0.5122384132626624</v>
       </c>
       <c r="B37" t="n">
-        <v>0.8213395358497312</v>
+        <v>0.5279915471428228</v>
       </c>
       <c r="C37" t="n">
-        <v>0.7343166531977483</v>
+        <v>0.7209105137940121</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0.5811611112380763</v>
+        <v>0.2309505297410821</v>
       </c>
       <c r="B38" t="n">
-        <v>0.143809484400736</v>
+        <v>0.3002793270342373</v>
       </c>
       <c r="C38" t="n">
-        <v>0.7929050434821922</v>
+        <v>0.4077142811209752</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0.01490735751349548</v>
+        <v>0.2558543814707607</v>
       </c>
       <c r="B39" t="n">
-        <v>0.6060360611120457</v>
+        <v>0.7732171472217509</v>
       </c>
       <c r="C39" t="n">
-        <v>0.1028898192868306</v>
+        <v>0.3941528907132671</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0.6275241993623608</v>
+        <v>0.04375137816752162</v>
       </c>
       <c r="B40" t="n">
-        <v>0.8744666296715237</v>
+        <v>0.1520945607530509</v>
       </c>
       <c r="C40" t="n">
-        <v>0.1549493097829708</v>
+        <v>0.5422311924200239</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0.9152558715280726</v>
+        <v>0.8647918938825606</v>
       </c>
       <c r="B41" t="n">
-        <v>0.7171111341377816</v>
+        <v>0.7290655622409506</v>
       </c>
       <c r="C41" t="n">
-        <v>0.7475359294106428</v>
+        <v>0.572864921759629</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0.6238723284428979</v>
+        <v>0.1860990387402971</v>
       </c>
       <c r="B42" t="n">
-        <v>0.6010499916092253</v>
+        <v>0.678861846714892</v>
       </c>
       <c r="C42" t="n">
-        <v>0.7699427791422706</v>
+        <v>0.2980343738247047</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>0.5865057474951278</v>
+        <v>0.2672894474930156</v>
       </c>
       <c r="B43" t="n">
-        <v>0.9669009739076477</v>
+        <v>0.3720575186245391</v>
       </c>
       <c r="C43" t="n">
-        <v>0.9700091903364031</v>
+        <v>0.9313810715562414</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0.03833701152874136</v>
+        <v>0.770292259023282</v>
       </c>
       <c r="B44" t="n">
-        <v>0.04257151638164414</v>
+        <v>0.2583880685245177</v>
       </c>
       <c r="C44" t="n">
-        <v>0.147454906647302</v>
+        <v>0.1868682889762991</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>0.3097565035019999</v>
+        <v>0.08100917428659771</v>
       </c>
       <c r="B45" t="n">
-        <v>0.7895025054196414</v>
+        <v>0.2953395106728386</v>
       </c>
       <c r="C45" t="n">
-        <v>0.07396661715164032</v>
+        <v>0.7343944729149134</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>0.4986884446399423</v>
+        <v>0.9665027359811725</v>
       </c>
       <c r="B46" t="n">
-        <v>0.07613370449555124</v>
+        <v>0.6988012345442296</v>
       </c>
       <c r="C46" t="n">
-        <v>0.374134317416882</v>
+        <v>0.2182317825273429</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>0.7509903544060018</v>
+        <v>0.9116615070499998</v>
       </c>
       <c r="B47" t="n">
-        <v>0.390725877801598</v>
+        <v>0.08001863490360639</v>
       </c>
       <c r="C47" t="n">
-        <v>0.9920154005484118</v>
+        <v>0.5401676017853347</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>0.3102747161369132</v>
+        <v>0.8823969174205619</v>
       </c>
       <c r="B48" t="n">
-        <v>0.9539419702647643</v>
+        <v>0.6072389278720315</v>
       </c>
       <c r="C48" t="n">
-        <v>0.4148525672197106</v>
+        <v>0.3261779900114073</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>0.2609394696353744</v>
+        <v>0.823394606613753</v>
       </c>
       <c r="B49" t="n">
-        <v>0.2033602181261845</v>
+        <v>0.3321195267510006</v>
       </c>
       <c r="C49" t="n">
-        <v>0.2106633111516826</v>
+        <v>0.7139611288852092</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>0.06848194258486628</v>
+        <v>0.09645102557224128</v>
       </c>
       <c r="B50" t="n">
-        <v>0.5117825548188787</v>
+        <v>0.5796199146727661</v>
       </c>
       <c r="C50" t="n">
-        <v>0.360035136504482</v>
+        <v>0.5838975994482817</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>0.07389641745171582</v>
+        <v>0.1169350056347902</v>
       </c>
       <c r="B51" t="n">
-        <v>0.6058779254595692</v>
+        <v>0.9181228233346993</v>
       </c>
       <c r="C51" t="n">
-        <v>0.981386317125416</v>
+        <v>0.9712946250912147</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>0.8465092083846327</v>
+        <v>0.4635817491242435</v>
       </c>
       <c r="B52" t="n">
-        <v>0.8563880815029496</v>
+        <v>0.7918784020799898</v>
       </c>
       <c r="C52" t="n">
-        <v>0.7288435814056341</v>
+        <v>0.9942683823550391</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>0.01153279182107125</v>
+        <v>0.1351812171402743</v>
       </c>
       <c r="B53" t="n">
-        <v>0.1146820485617625</v>
+        <v>0.2251953033657177</v>
       </c>
       <c r="C53" t="n">
-        <v>0.6215248689839324</v>
+        <v>0.2379865495956561</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>0.5880724289944242</v>
+        <v>0.639319317958832</v>
       </c>
       <c r="B54" t="n">
-        <v>0.7636254490732149</v>
+        <v>0.0621610245402322</v>
       </c>
       <c r="C54" t="n">
-        <v>0.01627112977904888</v>
+        <v>0.6438060460386765</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>0.5866666172816445</v>
+        <v>0.8507642594018884</v>
       </c>
       <c r="B55" t="n">
-        <v>0.9111529800061385</v>
+        <v>0.3184528638236247</v>
       </c>
       <c r="C55" t="n">
-        <v>0.3002927551251906</v>
+        <v>0.4322132118236727</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>0.6949964038120124</v>
+        <v>0.5416149354937224</v>
       </c>
       <c r="B56" t="n">
-        <v>0.5974241590378976</v>
+        <v>0.7522360084159545</v>
       </c>
       <c r="C56" t="n">
-        <v>0.4004718300337949</v>
+        <v>0.893066716307325</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0.7235369983580074</v>
+        <v>0.1050914265529587</v>
       </c>
       <c r="B57" t="n">
-        <v>0.7191303242018642</v>
+        <v>0.3673471699091158</v>
       </c>
       <c r="C57" t="n">
-        <v>0.2871744462250936</v>
+        <v>0.5046720553458034</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>0.3633969901312235</v>
+        <v>0.5024858340817442</v>
       </c>
       <c r="B58" t="n">
-        <v>0.9172604541112799</v>
+        <v>0.132044441782755</v>
       </c>
       <c r="C58" t="n">
-        <v>0.8435003334109284</v>
+        <v>0.9469741259974025</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0.4895783353837823</v>
+        <v>0.8939163146114611</v>
       </c>
       <c r="B59" t="n">
-        <v>0.2321353635935701</v>
+        <v>0.8679032307151948</v>
       </c>
       <c r="C59" t="n">
-        <v>0.7202638302157176</v>
+        <v>0.5897399814730381</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>0.7053619957612171</v>
+        <v>0.1587001561199497</v>
       </c>
       <c r="B60" t="n">
-        <v>0.2375369852595435</v>
+        <v>0.2082271662190525</v>
       </c>
       <c r="C60" t="n">
-        <v>0.405393611632455</v>
+        <v>0.8088448289583373</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>0.8538300092370983</v>
+        <v>0.7681652230339623</v>
       </c>
       <c r="B61" t="n">
-        <v>0.2066085584002203</v>
+        <v>0.1433754445969663</v>
       </c>
       <c r="C61" t="n">
-        <v>0.9081748605368657</v>
+        <v>0.7384281990390207</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>0.9082983746958826</v>
+        <v>0.3893757742051638</v>
       </c>
       <c r="B62" t="n">
-        <v>0.06253496433436279</v>
+        <v>0.667117977041053</v>
       </c>
       <c r="C62" t="n">
-        <v>0.4207414208318382</v>
+        <v>0.1554788224106896</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>0.3285644908358247</v>
+        <v>0.6767309085072258</v>
       </c>
       <c r="B63" t="n">
-        <v>0.8204021168104364</v>
+        <v>0.3710839112739485</v>
       </c>
       <c r="C63" t="n">
-        <v>0.3646599105476749</v>
+        <v>0.9167986390477413</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>0.6544621625267422</v>
+        <v>0.03489720309147959</v>
       </c>
       <c r="B64" t="n">
-        <v>0.02843593241125186</v>
+        <v>0.8549331212974479</v>
       </c>
       <c r="C64" t="n">
-        <v>0.3034714405646229</v>
+        <v>0.9699439655038631</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>0.5292214027902119</v>
+        <v>0.07208670368883863</v>
       </c>
       <c r="B65" t="n">
-        <v>0.2111129104633749</v>
+        <v>0.3175030631629501</v>
       </c>
       <c r="C65" t="n">
-        <v>0.6602755484034684</v>
+        <v>0.9478562085457171</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>0.2818677793245959</v>
+        <v>0.2943624614894379</v>
       </c>
       <c r="B66" t="n">
-        <v>0.3256735370271887</v>
+        <v>0.701533771858631</v>
       </c>
       <c r="C66" t="n">
-        <v>0.5443091656954412</v>
+        <v>0.1883553048960026</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>0.3746323596506181</v>
+        <v>0.5149035361048779</v>
       </c>
       <c r="B67" t="n">
-        <v>0.9791351820746447</v>
+        <v>0.3193375226806798</v>
       </c>
       <c r="C67" t="n">
-        <v>0.04970690246490961</v>
+        <v>0.3070305873588572</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>0.9144445164286367</v>
+        <v>0.1810091478887484</v>
       </c>
       <c r="B68" t="n">
-        <v>0.514408175164793</v>
+        <v>0.05314872085997668</v>
       </c>
       <c r="C68" t="n">
-        <v>0.9361996647262589</v>
+        <v>0.4915425718239567</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>0.6587898875591197</v>
+        <v>0.4969534255443565</v>
       </c>
       <c r="B69" t="n">
-        <v>0.5316091001707469</v>
+        <v>0.8206747279068564</v>
       </c>
       <c r="C69" t="n">
-        <v>0.639346980642726</v>
+        <v>0.7956090918747634</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>0.02482745859624447</v>
+        <v>0.6550326165097876</v>
       </c>
       <c r="B70" t="n">
-        <v>0.9124674744403649</v>
+        <v>0.1296753818120929</v>
       </c>
       <c r="C70" t="n">
-        <v>0.07691315457055958</v>
+        <v>0.8159278163928425</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>0.05094330177438777</v>
+        <v>0.4964843660326866</v>
       </c>
       <c r="B71" t="n">
-        <v>0.006641393876438029</v>
+        <v>0.4745421765275007</v>
       </c>
       <c r="C71" t="n">
-        <v>0.615686935169707</v>
+        <v>0.711063269274919</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>0.5226602724339653</v>
+        <v>0.9766385397549184</v>
       </c>
       <c r="B72" t="n">
-        <v>0.165559841228719</v>
+        <v>0.4044272146242874</v>
       </c>
       <c r="C72" t="n">
-        <v>0.6661009006498859</v>
+        <v>0.2942097423468787</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>0.3413514367128164</v>
+        <v>0.8886424986444345</v>
       </c>
       <c r="B73" t="n">
-        <v>0.5744471951975323</v>
+        <v>0.5881012460990366</v>
       </c>
       <c r="C73" t="n">
-        <v>0.6471435084348885</v>
+        <v>0.4822348060089867</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>0.1652839158680404</v>
+        <v>0.5184669381152722</v>
       </c>
       <c r="B74" t="n">
-        <v>0.2206459082457382</v>
+        <v>0.3543617158218179</v>
       </c>
       <c r="C74" t="n">
-        <v>0.4774214807965127</v>
+        <v>0.1485785159311721</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>0.2654916453268901</v>
+        <v>0.7269539352385755</v>
       </c>
       <c r="B75" t="n">
-        <v>0.5387258440494344</v>
+        <v>0.3245817427165039</v>
       </c>
       <c r="C75" t="n">
-        <v>0.2622836128739298</v>
+        <v>0.6491679148356999</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>0.3044067846218442</v>
+        <v>0.4457610303688275</v>
       </c>
       <c r="B76" t="n">
-        <v>0.163965115314367</v>
+        <v>0.5363397646017874</v>
       </c>
       <c r="C76" t="n">
-        <v>0.4189384082170772</v>
+        <v>0.2505456234253118</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>0.516828484703505</v>
+        <v>0.3106066232825615</v>
       </c>
       <c r="B77" t="n">
-        <v>0.03640224883117804</v>
+        <v>0.09233252522802526</v>
       </c>
       <c r="C77" t="n">
-        <v>0.5279291746234993</v>
+        <v>0.8019430454280457</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>0.9440100970536093</v>
+        <v>0.5211703545203038</v>
       </c>
       <c r="B78" t="n">
-        <v>0.6647400701906468</v>
+        <v>0.4937114295001336</v>
       </c>
       <c r="C78" t="n">
-        <v>0.6500675492846409</v>
+        <v>0.880763092175325</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>0.8461255050627124</v>
+        <v>0.2936438128189832</v>
       </c>
       <c r="B79" t="n">
-        <v>0.6080869741648586</v>
+        <v>0.6879045228957242</v>
       </c>
       <c r="C79" t="n">
-        <v>0.5945276381837437</v>
+        <v>0.2201823859487426</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>0.7442235895628793</v>
+        <v>0.3839456081605973</v>
       </c>
       <c r="B80" t="n">
-        <v>0.6019428291986827</v>
+        <v>0.7740744703763949</v>
       </c>
       <c r="C80" t="n">
-        <v>0.1634936297027978</v>
+        <v>0.8478163231251566</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>0.0884073017430993</v>
+        <v>0.7903950190403362</v>
       </c>
       <c r="B81" t="n">
-        <v>0.4806508876899199</v>
+        <v>0.6508037115466462</v>
       </c>
       <c r="C81" t="n">
-        <v>0.4061061209680594</v>
+        <v>0.8889897550733081</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>0.04739944177791278</v>
+        <v>0.1627946153365623</v>
       </c>
       <c r="B82" t="n">
-        <v>0.482128863395005</v>
+        <v>0.4643825912248726</v>
       </c>
       <c r="C82" t="n">
-        <v>0.1761866458416728</v>
+        <v>0.3231738403238572</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>0.7742691393297866</v>
+        <v>0.8516363705588597</v>
       </c>
       <c r="B83" t="n">
-        <v>0.09849416407379918</v>
+        <v>0.9164942114467742</v>
       </c>
       <c r="C83" t="n">
-        <v>0.6028461007445748</v>
+        <v>0.9940997320270676</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>0.976817422548874</v>
+        <v>0.578618223652045</v>
       </c>
       <c r="B84" t="n">
-        <v>0.1054955249317705</v>
+        <v>0.4179536733685759</v>
       </c>
       <c r="C84" t="n">
-        <v>0.05433015965492749</v>
+        <v>0.7283774774850734</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>0.7792835462157338</v>
+        <v>0.07146350781043842</v>
       </c>
       <c r="B85" t="n">
-        <v>0.08154996817450832</v>
+        <v>0.7538178944472897</v>
       </c>
       <c r="C85" t="n">
-        <v>0.6332726558430962</v>
+        <v>0.4353957080558639</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>0.2230250544351123</v>
+        <v>0.9350234525379962</v>
       </c>
       <c r="B86" t="n">
-        <v>0.3028531131114703</v>
+        <v>0.2029686241321239</v>
       </c>
       <c r="C86" t="n">
-        <v>0.5762342593702303</v>
+        <v>0.9453079146861429</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>0.07077221103619535</v>
+        <v>0.3941496602074946</v>
       </c>
       <c r="B87" t="n">
-        <v>0.8442969707477175</v>
+        <v>0.9306411172826856</v>
       </c>
       <c r="C87" t="n">
-        <v>0.7557455441114868</v>
+        <v>0.1799248044267657</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>0.7624798194857603</v>
+        <v>0.7157188250942534</v>
       </c>
       <c r="B88" t="n">
-        <v>0.005619446966691477</v>
+        <v>0.3542437345992165</v>
       </c>
       <c r="C88" t="n">
-        <v>0.1470650295023141</v>
+        <v>0.8552053170642878</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>0.08159640091224118</v>
+        <v>0.05212695734308359</v>
       </c>
       <c r="B89" t="n">
-        <v>0.35378142172709</v>
+        <v>0.5618055880113517</v>
       </c>
       <c r="C89" t="n">
-        <v>0.3327169247637144</v>
+        <v>0.0603421569177508</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>0.08312374131942024</v>
+        <v>0.2369466851270258</v>
       </c>
       <c r="B90" t="n">
-        <v>0.4866761084815573</v>
+        <v>0.4155398900534286</v>
       </c>
       <c r="C90" t="n">
-        <v>0.9759230762027176</v>
+        <v>0.7159862303151486</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>0.3376522934532856</v>
+        <v>0.4645734127804664</v>
       </c>
       <c r="B91" t="n">
-        <v>0.6207943528145153</v>
+        <v>0.2250908996478669</v>
       </c>
       <c r="C91" t="n">
-        <v>0.7420775218057759</v>
+        <v>0.8773191864458413</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0.2623784266731283</v>
+        <v>0.3965856510387251</v>
       </c>
       <c r="B92" t="n">
-        <v>0.02897363052539981</v>
+        <v>0.2770626591620254</v>
       </c>
       <c r="C92" t="n">
-        <v>0.9983212546975793</v>
+        <v>0.8763600240689823</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>0.1250386486135606</v>
+        <v>0.540405212040195</v>
       </c>
       <c r="B93" t="n">
-        <v>0.05368716356050485</v>
+        <v>0.379165250233039</v>
       </c>
       <c r="C93" t="n">
-        <v>0.005564042671999836</v>
+        <v>0.8745527654242466</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>0.1287640922354498</v>
+        <v>0.9416386881017255</v>
       </c>
       <c r="B94" t="n">
-        <v>0.2849134738827467</v>
+        <v>0.1679685085570363</v>
       </c>
       <c r="C94" t="n">
-        <v>0.1572693211713843</v>
+        <v>0.3716302140785965</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>0.0322588680417184</v>
+        <v>0.5020026259790688</v>
       </c>
       <c r="B95" t="n">
-        <v>0.4568667272725655</v>
+        <v>0.8348990767311817</v>
       </c>
       <c r="C95" t="n">
-        <v>0.1029800520751066</v>
+        <v>0.865982663413316</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>0.5986294488977343</v>
+        <v>0.3666016662544316</v>
       </c>
       <c r="B96" t="n">
-        <v>0.7702147889700345</v>
+        <v>0.1474795027860196</v>
       </c>
       <c r="C96" t="n">
-        <v>0.4620297476448655</v>
+        <v>0.8288396867948219</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>0.02859077447658454</v>
+        <v>0.2269651200852236</v>
       </c>
       <c r="B97" t="n">
-        <v>0.9046826469812204</v>
+        <v>0.2516599687949611</v>
       </c>
       <c r="C97" t="n">
-        <v>0.8053002655881362</v>
+        <v>0.3108526510245896</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>0.8479811016648608</v>
+        <v>0.6586540905034437</v>
       </c>
       <c r="B98" t="n">
-        <v>0.1441874731668519</v>
+        <v>0.7708474677142754</v>
       </c>
       <c r="C98" t="n">
-        <v>0.6181742472944491</v>
+        <v>0.4197523026144331</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>0.7148047934091549</v>
+        <v>0.8566340214548899</v>
       </c>
       <c r="B99" t="n">
-        <v>0.7990022064902437</v>
+        <v>0.5542881314698378</v>
       </c>
       <c r="C99" t="n">
-        <v>0.2882897343693059</v>
+        <v>0.7537607364185965</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>0.6783241821173379</v>
+        <v>0.05870420473629145</v>
       </c>
       <c r="B100" t="n">
-        <v>0.7729031818347517</v>
+        <v>0.988645517212568</v>
       </c>
       <c r="C100" t="n">
-        <v>0.9189980996599203</v>
+        <v>0.5062514734827349</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>0.105686207055654</v>
+        <v>0.1439141791287202</v>
       </c>
       <c r="B101" t="n">
-        <v>0.2750472467928942</v>
+        <v>0.4650613920021659</v>
       </c>
       <c r="C101" t="n">
-        <v>0.1358365723022025</v>
+        <v>0.5872963238083758</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added unified excel and resumen graph
</commit_message>
<xml_diff>
--- a/datos/invalido.xlsx
+++ b/datos/invalido.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="datos_IV" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,1102 +436,1138 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.3642610991371413</v>
+        <v>0.9874990127998821</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4393585701914053</v>
+        <v>0.06677024569169943</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8622101811175628</v>
+        <v>0.2665554431904881</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.4347973968947693</v>
+        <v>0.2388237818088111</v>
       </c>
       <c r="B3" t="n">
-        <v>0.2629513920687184</v>
+        <v>0.3644702894730326</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7144550027917037</v>
+        <v>0.2973896512244831</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.9534742846485205</v>
+        <v>0.3050919281643729</v>
       </c>
       <c r="B4" t="n">
-        <v>0.7478364194288035</v>
+        <v>0.5016238019191793</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5535501018671309</v>
+        <v>0.5982253971921958</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.4869342562026893</v>
+        <v>0.5893571991659903</v>
       </c>
       <c r="B5" t="n">
-        <v>0.3946206049615253</v>
+        <v>0.9753072458117519</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8686273284224302</v>
+        <v>0.2936853618077935</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.8459623319139834</v>
+        <v>0.9770542941144075</v>
       </c>
       <c r="B6" t="n">
-        <v>0.7150521764798419</v>
+        <v>0.2644880094674655</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9841353262407144</v>
+        <v>0.7312704729336752</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.521491098019836</v>
+        <v>0.479376438723084</v>
       </c>
       <c r="B7" t="n">
-        <v>0.5536828506031738</v>
+        <v>0.1537303662587997</v>
       </c>
       <c r="C7" t="n">
-        <v>0.08590297473869524</v>
+        <v>0.5310391009584273</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.2574839709447263</v>
+        <v>0.01024244589268164</v>
       </c>
       <c r="B8" t="n">
-        <v>0.935439306848471</v>
+        <v>0.4273069704966358</v>
       </c>
       <c r="C8" t="n">
-        <v>0.362206318327155</v>
+        <v>0.2509619025382051</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.3109414981373435</v>
+        <v>0.4393441084250733</v>
       </c>
       <c r="B9" t="n">
-        <v>0.3531859871489232</v>
+        <v>0.3992231954336198</v>
       </c>
       <c r="C9" t="n">
-        <v>0.590760023730611</v>
+        <v>0.7145852070423722</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.9235485709030722</v>
+        <v>0.2589031414636561</v>
       </c>
       <c r="B10" t="n">
-        <v>0.819959338137869</v>
+        <v>0.6519621509920489</v>
       </c>
       <c r="C10" t="n">
-        <v>0.3310786663202981</v>
+        <v>0.5224100931491077</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.132501577462024</v>
+        <v>0.2690526979631466</v>
       </c>
       <c r="B11" t="n">
-        <v>0.4361854078553131</v>
+        <v>0.4340598945304858</v>
       </c>
       <c r="C11" t="n">
-        <v>0.6908893957816845</v>
+        <v>0.1108373374869082</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.1579645997602448</v>
+        <v>0.4074904313410578</v>
       </c>
       <c r="B12" t="n">
-        <v>0.6153441821266217</v>
+        <v>0.6601740546215746</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9547386496628771</v>
+        <v>0.05066345295299102</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.8234611284095843</v>
+        <v>0.01263216377339582</v>
       </c>
       <c r="B13" t="n">
-        <v>0.5489742525658842</v>
+        <v>0.9442493643381097</v>
       </c>
       <c r="C13" t="n">
-        <v>0.6788943206172632</v>
+        <v>0.1898554221429157</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.4865046164693585</v>
+        <v>0.4452917391190032</v>
       </c>
       <c r="B14" t="n">
-        <v>0.6198293260246734</v>
+        <v>0.666445767462321</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3273554218327915</v>
+        <v>0.05432948087139311</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.2081017281585414</v>
+        <v>0.7448109679154249</v>
       </c>
       <c r="B15" t="n">
-        <v>0.4742407635052142</v>
+        <v>0.2381676162995129</v>
       </c>
       <c r="C15" t="n">
-        <v>0.7714495235733287</v>
+        <v>0.1293077380396909</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.9469235121667602</v>
+        <v>0.8174211373906262</v>
       </c>
       <c r="B16" t="n">
-        <v>0.9312617306730616</v>
+        <v>0.8780432264562372</v>
       </c>
       <c r="C16" t="n">
-        <v>0.9827423910189745</v>
+        <v>0.1627470783819276</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.7461168377830257</v>
+        <v>0.1884631800717324</v>
       </c>
       <c r="B17" t="n">
-        <v>0.1550816135569292</v>
+        <v>0.04735892516134632</v>
       </c>
       <c r="C17" t="n">
-        <v>0.3824229237223835</v>
+        <v>0.1185656979684888</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.913182090289098</v>
+        <v>0.4413567116996301</v>
       </c>
       <c r="B18" t="n">
-        <v>0.7652182636758874</v>
+        <v>0.06694037429760646</v>
       </c>
       <c r="C18" t="n">
-        <v>0.6719487440962053</v>
+        <v>0.09713214054092689</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.4725751022167024</v>
+        <v>0.03480931082092131</v>
       </c>
       <c r="B19" t="n">
-        <v>0.1584509778857712</v>
+        <v>0.7065353382231385</v>
       </c>
       <c r="C19" t="n">
-        <v>0.7813754559820908</v>
+        <v>0.1664474371930433</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.1103366307018246</v>
+        <v>0.7326836773809215</v>
       </c>
       <c r="B20" t="n">
-        <v>0.3394823663165598</v>
+        <v>0.4348324619608551</v>
       </c>
       <c r="C20" t="n">
-        <v>0.4509238652293436</v>
+        <v>0.1072374619591839</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.903295924411914</v>
+        <v>0.4720373484705401</v>
       </c>
       <c r="B21" t="n">
-        <v>0.9752387379495151</v>
+        <v>0.3909408577436195</v>
       </c>
       <c r="C21" t="n">
-        <v>0.18661260434781</v>
+        <v>0.7083105901485033</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.513642651131759</v>
+        <v>0.443832390624036</v>
       </c>
       <c r="B22" t="n">
-        <v>0.2908779126374178</v>
+        <v>0.2629954382586027</v>
       </c>
       <c r="C22" t="n">
-        <v>0.2416513763615679</v>
+        <v>0.6669224873693664</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.3611804801943612</v>
+        <v>0.1439480694055761</v>
       </c>
       <c r="B23" t="n">
-        <v>0.5605522801558406</v>
+        <v>0.4905282806678342</v>
       </c>
       <c r="C23" t="n">
-        <v>0.1913218371920437</v>
+        <v>0.4629617156877679</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0.9730203588687899</v>
+        <v>0.1228364865866441</v>
       </c>
       <c r="B24" t="n">
-        <v>0.4110373957826468</v>
+        <v>0.5157355580453774</v>
       </c>
       <c r="C24" t="n">
-        <v>0.7555646816097903</v>
+        <v>0.9138160004779783</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.323971971426414</v>
+        <v>0.5886803983603418</v>
       </c>
       <c r="B25" t="n">
-        <v>0.1669673928923394</v>
+        <v>0.3041980602616896</v>
       </c>
       <c r="C25" t="n">
-        <v>0.509330040650285</v>
+        <v>0.5590818551178421</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.2996228984082996</v>
+        <v>0.954356730712049</v>
       </c>
       <c r="B26" t="n">
-        <v>0.5661809512956646</v>
+        <v>0.527900199790815</v>
       </c>
       <c r="C26" t="n">
-        <v>0.6833075525779972</v>
+        <v>0.5730853456973594</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0.875993506445928</v>
+        <v>0.3317823811311988</v>
       </c>
       <c r="B27" t="n">
-        <v>0.9558902765282056</v>
+        <v>0.4966460769845048</v>
       </c>
       <c r="C27" t="n">
-        <v>0.4332152602491856</v>
+        <v>0.3335328384446756</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.718793588379087</v>
+        <v>0.2141317598304335</v>
       </c>
       <c r="B28" t="n">
-        <v>0.3547906747599755</v>
+        <v>0.5273979514287739</v>
       </c>
       <c r="C28" t="n">
-        <v>0.5888230144390761</v>
+        <v>0.4618722760680001</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.6485937629614191</v>
+        <v>0.7137165311009247</v>
       </c>
       <c r="B29" t="n">
-        <v>0.195819452171565</v>
+        <v>0.781676670344297</v>
       </c>
       <c r="C29" t="n">
-        <v>0.4617002665334933</v>
+        <v>0.2520191911371871</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0.3208788751497276</v>
+        <v>0.3903534799255833</v>
       </c>
       <c r="B30" t="n">
-        <v>0.8347857258514697</v>
+        <v>0.4807009863521372</v>
       </c>
       <c r="C30" t="n">
-        <v>0.8261047130838384</v>
+        <v>0.4215107891300273</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0.4486368693960292</v>
+        <v>0.5036426005611084</v>
       </c>
       <c r="B31" t="n">
-        <v>0.6076980897217376</v>
+        <v>0.6008560126366141</v>
       </c>
       <c r="C31" t="n">
-        <v>0.1852126749486049</v>
+        <v>0.9022739024331301</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0.1434360931386645</v>
+        <v>0.1307122580442486</v>
       </c>
       <c r="B32" t="n">
-        <v>0.3310285579544189</v>
+        <v>0.3427939867750914</v>
       </c>
       <c r="C32" t="n">
-        <v>0.6490133912500426</v>
+        <v>0.04367675420169359</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0.8732318620256962</v>
+        <v>0.4509891456417698</v>
       </c>
       <c r="B33" t="n">
-        <v>0.1044027230703831</v>
+        <v>0.6164939960438991</v>
       </c>
       <c r="C33" t="n">
-        <v>0.5947777887979242</v>
+        <v>0.8047732035683186</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0.8993338208758763</v>
+        <v>0.5583162033383633</v>
       </c>
       <c r="B34" t="n">
-        <v>0.1529107547971765</v>
+        <v>0.3651597013411998</v>
       </c>
       <c r="C34" t="n">
-        <v>0.7676449816146649</v>
+        <v>0.9485533932068574</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.9325048043806701</v>
+        <v>0.9557673144305362</v>
       </c>
       <c r="B35" t="n">
-        <v>0.9684686112713446</v>
+        <v>0.6522274209009953</v>
       </c>
       <c r="C35" t="n">
-        <v>0.06020398441737773</v>
+        <v>0.5471894514894651</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0.7917744936645598</v>
+        <v>0.9286703506782776</v>
       </c>
       <c r="B36" t="n">
-        <v>0.3186336153903198</v>
+        <v>0.3903454228998762</v>
       </c>
       <c r="C36" t="n">
-        <v>0.6465507270531345</v>
+        <v>0.04150677825622229</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0.5122384132626624</v>
+        <v>0.794431496367475</v>
       </c>
       <c r="B37" t="n">
-        <v>0.5279915471428228</v>
+        <v>0.829008796899282</v>
       </c>
       <c r="C37" t="n">
-        <v>0.7209105137940121</v>
+        <v>0.733804353195317</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0.2309505297410821</v>
+        <v>0.1815392058259165</v>
       </c>
       <c r="B38" t="n">
-        <v>0.3002793270342373</v>
+        <v>0.7475658591889965</v>
       </c>
       <c r="C38" t="n">
-        <v>0.4077142811209752</v>
+        <v>0.3481803706181332</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0.2558543814707607</v>
+        <v>0.505073008331598</v>
       </c>
       <c r="B39" t="n">
-        <v>0.7732171472217509</v>
+        <v>0.6513286354644205</v>
       </c>
       <c r="C39" t="n">
-        <v>0.3941528907132671</v>
+        <v>0.1999644143083077</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0.04375137816752162</v>
+        <v>0.5714456660839959</v>
       </c>
       <c r="B40" t="n">
-        <v>0.1520945607530509</v>
+        <v>0.07333036234829726</v>
       </c>
       <c r="C40" t="n">
-        <v>0.5422311924200239</v>
+        <v>0.6169999844912766</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0.8647918938825606</v>
+        <v>0.8602212316519979</v>
       </c>
       <c r="B41" t="n">
-        <v>0.7290655622409506</v>
+        <v>0.4557838728783645</v>
       </c>
       <c r="C41" t="n">
-        <v>0.572864921759629</v>
+        <v>0.7141898750246499</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0.1860990387402971</v>
+        <v>0.07603086028357309</v>
       </c>
       <c r="B42" t="n">
-        <v>0.678861846714892</v>
+        <v>0.004790890494288158</v>
       </c>
       <c r="C42" t="n">
-        <v>0.2980343738247047</v>
+        <v>0.1819494312673533</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>0.2672894474930156</v>
+        <v>0.8515313585389757</v>
       </c>
       <c r="B43" t="n">
-        <v>0.3720575186245391</v>
+        <v>0.5698585044961687</v>
       </c>
       <c r="C43" t="n">
-        <v>0.9313810715562414</v>
+        <v>0.01907692554616769</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0.770292259023282</v>
+        <v>0.801913266514057</v>
       </c>
       <c r="B44" t="n">
-        <v>0.2583880685245177</v>
+        <v>0.6513491755660888</v>
       </c>
       <c r="C44" t="n">
-        <v>0.1868682889762991</v>
+        <v>0.9253015555885107</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>0.08100917428659771</v>
+        <v>0.7640316172419207</v>
       </c>
       <c r="B45" t="n">
-        <v>0.2953395106728386</v>
+        <v>0.8035953509595312</v>
       </c>
       <c r="C45" t="n">
-        <v>0.7343944729149134</v>
+        <v>0.02320126816109913</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>0.9665027359811725</v>
+        <v>0.7984096165759804</v>
       </c>
       <c r="B46" t="n">
-        <v>0.6988012345442296</v>
+        <v>0.5677980066242363</v>
       </c>
       <c r="C46" t="n">
-        <v>0.2182317825273429</v>
+        <v>0.9140885085177074</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>0.9116615070499998</v>
+        <v>0.1729136964134047</v>
       </c>
       <c r="B47" t="n">
-        <v>0.08001863490360639</v>
+        <v>0.05906188779167776</v>
       </c>
       <c r="C47" t="n">
-        <v>0.5401676017853347</v>
+        <v>0.1077812565998842</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>0.8823969174205619</v>
+        <v>0.1402759994779184</v>
       </c>
       <c r="B48" t="n">
-        <v>0.6072389278720315</v>
+        <v>0.01805473731272422</v>
       </c>
       <c r="C48" t="n">
-        <v>0.3261779900114073</v>
+        <v>0.3309753883496311</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>0.823394606613753</v>
+        <v>0.6756312800527787</v>
       </c>
       <c r="B49" t="n">
-        <v>0.3321195267510006</v>
+        <v>0.1253877524561836</v>
       </c>
       <c r="C49" t="n">
-        <v>0.7139611288852092</v>
+        <v>0.7766219008113427</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>0.09645102557224128</v>
+        <v>0.8209761339297081</v>
       </c>
       <c r="B50" t="n">
-        <v>0.5796199146727661</v>
+        <v>0.4714541273419459</v>
       </c>
       <c r="C50" t="n">
-        <v>0.5838975994482817</v>
+        <v>0.5167524465358665</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>0.1169350056347902</v>
+        <v>0.905691676608396</v>
       </c>
       <c r="B51" t="n">
-        <v>0.9181228233346993</v>
+        <v>0.9853987232100184</v>
       </c>
       <c r="C51" t="n">
-        <v>0.9712946250912147</v>
+        <v>0.4908377224614123</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>0.4635817491242435</v>
+        <v>0.4642070887283199</v>
       </c>
       <c r="B52" t="n">
-        <v>0.7918784020799898</v>
+        <v>0.6606933194687443</v>
       </c>
       <c r="C52" t="n">
-        <v>0.9942683823550391</v>
+        <v>0.4826751854862502</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>0.1351812171402743</v>
+        <v>0.5604805953091815</v>
       </c>
       <c r="B53" t="n">
-        <v>0.2251953033657177</v>
+        <v>0.5208140655215029</v>
       </c>
       <c r="C53" t="n">
-        <v>0.2379865495956561</v>
+        <v>0.2147992869204706</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>0.639319317958832</v>
+        <v>0.938688760365186</v>
       </c>
       <c r="B54" t="n">
-        <v>0.0621610245402322</v>
+        <v>0.4416779004996486</v>
       </c>
       <c r="C54" t="n">
-        <v>0.6438060460386765</v>
+        <v>0.1828624202464506</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>0.8507642594018884</v>
+        <v>0.2982024906131185</v>
       </c>
       <c r="B55" t="n">
-        <v>0.3184528638236247</v>
+        <v>0.4349468235591191</v>
       </c>
       <c r="C55" t="n">
-        <v>0.4322132118236727</v>
+        <v>0.8177461579390259</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>0.5416149354937224</v>
+        <v>0.8470913140247939</v>
       </c>
       <c r="B56" t="n">
-        <v>0.7522360084159545</v>
+        <v>0.7359634538787764</v>
       </c>
       <c r="C56" t="n">
-        <v>0.893066716307325</v>
+        <v>0.7223571479737906</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0.1050914265529587</v>
+        <v>0.3770349214107344</v>
       </c>
       <c r="B57" t="n">
-        <v>0.3673471699091158</v>
+        <v>0.2509027047230528</v>
       </c>
       <c r="C57" t="n">
-        <v>0.5046720553458034</v>
+        <v>0.171899524453926</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>0.5024858340817442</v>
+        <v>0.2344235574784733</v>
       </c>
       <c r="B58" t="n">
-        <v>0.132044441782755</v>
+        <v>0.1670255367589518</v>
       </c>
       <c r="C58" t="n">
-        <v>0.9469741259974025</v>
+        <v>0.926446297842725</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0.8939163146114611</v>
+        <v>0.226059756807948</v>
       </c>
       <c r="B59" t="n">
-        <v>0.8679032307151948</v>
+        <v>0.5596307523515082</v>
       </c>
       <c r="C59" t="n">
-        <v>0.5897399814730381</v>
+        <v>0.134383605127593</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>0.1587001561199497</v>
+        <v>0.1572370660524939</v>
       </c>
       <c r="B60" t="n">
-        <v>0.2082271662190525</v>
+        <v>0.2552190524356569</v>
       </c>
       <c r="C60" t="n">
-        <v>0.8088448289583373</v>
+        <v>0.7732997735376504</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>0.7681652230339623</v>
+        <v>0.5083943095958892</v>
       </c>
       <c r="B61" t="n">
-        <v>0.1433754445969663</v>
+        <v>0.5273289792025656</v>
       </c>
       <c r="C61" t="n">
-        <v>0.7384281990390207</v>
+        <v>0.1324522948412756</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>0.3893757742051638</v>
+        <v>0.3536394148777138</v>
       </c>
       <c r="B62" t="n">
-        <v>0.667117977041053</v>
+        <v>0.4061293644955662</v>
       </c>
       <c r="C62" t="n">
-        <v>0.1554788224106896</v>
+        <v>0.9480931985175357</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>0.6767309085072258</v>
+        <v>0.5006586758817577</v>
       </c>
       <c r="B63" t="n">
-        <v>0.3710839112739485</v>
+        <v>0.7431316060361215</v>
       </c>
       <c r="C63" t="n">
-        <v>0.9167986390477413</v>
+        <v>0.1653076892731024</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>0.03489720309147959</v>
+        <v>0.02743917099881232</v>
       </c>
       <c r="B64" t="n">
-        <v>0.8549331212974479</v>
+        <v>0.7063329687263883</v>
       </c>
       <c r="C64" t="n">
-        <v>0.9699439655038631</v>
+        <v>0.7769559657261144</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>0.07208670368883863</v>
+        <v>0.008601315338603421</v>
       </c>
       <c r="B65" t="n">
-        <v>0.3175030631629501</v>
+        <v>0.5585341385773461</v>
       </c>
       <c r="C65" t="n">
-        <v>0.9478562085457171</v>
+        <v>0.4796076850792853</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>0.2943624614894379</v>
+        <v>0.1895783139464038</v>
       </c>
       <c r="B66" t="n">
-        <v>0.701533771858631</v>
+        <v>0.5749277824358836</v>
       </c>
       <c r="C66" t="n">
-        <v>0.1883553048960026</v>
+        <v>0.9928837026206382</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>0.5149035361048779</v>
+        <v>0.09225991059377914</v>
       </c>
       <c r="B67" t="n">
-        <v>0.3193375226806798</v>
+        <v>0.5885909911203842</v>
       </c>
       <c r="C67" t="n">
-        <v>0.3070305873588572</v>
+        <v>0.6251888247834982</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>0.1810091478887484</v>
+        <v>0.6360112996251258</v>
       </c>
       <c r="B68" t="n">
-        <v>0.05314872085997668</v>
+        <v>0.2571596601591882</v>
       </c>
       <c r="C68" t="n">
-        <v>0.4915425718239567</v>
+        <v>0.629905414278205</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>0.4969534255443565</v>
+        <v>0.5130992426379457</v>
       </c>
       <c r="B69" t="n">
-        <v>0.8206747279068564</v>
+        <v>0.138061914930562</v>
       </c>
       <c r="C69" t="n">
-        <v>0.7956090918747634</v>
+        <v>0.9669262265359706</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>0.6550326165097876</v>
+        <v>0.4168409486242288</v>
       </c>
       <c r="B70" t="n">
-        <v>0.1296753818120929</v>
+        <v>0.3600503949618424</v>
       </c>
       <c r="C70" t="n">
-        <v>0.8159278163928425</v>
+        <v>0.2691073253382498</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>0.4964843660326866</v>
+        <v>0.3333525013620574</v>
       </c>
       <c r="B71" t="n">
-        <v>0.4745421765275007</v>
+        <v>0.2241353863301019</v>
       </c>
       <c r="C71" t="n">
-        <v>0.711063269274919</v>
+        <v>0.709533632455761</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>0.9766385397549184</v>
+        <v>0.7284142279543322</v>
       </c>
       <c r="B72" t="n">
-        <v>0.4044272146242874</v>
+        <v>0.8317693664008753</v>
       </c>
       <c r="C72" t="n">
-        <v>0.2942097423468787</v>
+        <v>0.9677727941362805</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>0.8886424986444345</v>
+        <v>0.4758014732974662</v>
       </c>
       <c r="B73" t="n">
-        <v>0.5881012460990366</v>
+        <v>0.9568405042265429</v>
       </c>
       <c r="C73" t="n">
-        <v>0.4822348060089867</v>
+        <v>0.5214652776837124</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>0.5184669381152722</v>
+        <v>0.004653297983023497</v>
       </c>
       <c r="B74" t="n">
-        <v>0.3543617158218179</v>
+        <v>0.8513361245215952</v>
       </c>
       <c r="C74" t="n">
-        <v>0.1485785159311721</v>
+        <v>0.4668138625687197</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>0.7269539352385755</v>
+        <v>0.8573585571466749</v>
       </c>
       <c r="B75" t="n">
-        <v>0.3245817427165039</v>
+        <v>0.189836056649563</v>
       </c>
       <c r="C75" t="n">
-        <v>0.6491679148356999</v>
+        <v>0.250158645183762</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>0.4457610303688275</v>
+        <v>0.149097494404173</v>
       </c>
       <c r="B76" t="n">
-        <v>0.5363397646017874</v>
+        <v>0.3730386166454077</v>
       </c>
       <c r="C76" t="n">
-        <v>0.2505456234253118</v>
+        <v>0.8946570922620906</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>0.3106066232825615</v>
+        <v>0.219750772513014</v>
       </c>
       <c r="B77" t="n">
-        <v>0.09233252522802526</v>
+        <v>0.08625911728143343</v>
       </c>
       <c r="C77" t="n">
-        <v>0.8019430454280457</v>
+        <v>0.2364085437380137</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>0.5211703545203038</v>
+        <v>0.7098255003228924</v>
       </c>
       <c r="B78" t="n">
-        <v>0.4937114295001336</v>
+        <v>0.007694803654728077</v>
       </c>
       <c r="C78" t="n">
-        <v>0.880763092175325</v>
+        <v>0.04331740923028216</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>0.2936438128189832</v>
+        <v>0.4030171688909681</v>
       </c>
       <c r="B79" t="n">
-        <v>0.6879045228957242</v>
+        <v>0.03676875800067925</v>
       </c>
       <c r="C79" t="n">
-        <v>0.2201823859487426</v>
+        <v>0.4405246459158451</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>0.3839456081605973</v>
+        <v>0.212488691392695</v>
       </c>
       <c r="B80" t="n">
-        <v>0.7740744703763949</v>
+        <v>0.1097826359017032</v>
       </c>
       <c r="C80" t="n">
-        <v>0.8478163231251566</v>
+        <v>0.04371226099423831</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>0.7903950190403362</v>
+        <v>0.1311048574922197</v>
       </c>
       <c r="B81" t="n">
-        <v>0.6508037115466462</v>
+        <v>0.9331847436861107</v>
       </c>
       <c r="C81" t="n">
-        <v>0.8889897550733081</v>
+        <v>0.980219322082783</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>0.1627946153365623</v>
+        <v>0.2383600704728631</v>
       </c>
       <c r="B82" t="n">
-        <v>0.4643825912248726</v>
+        <v>0.1211941230774263</v>
       </c>
       <c r="C82" t="n">
-        <v>0.3231738403238572</v>
+        <v>0.9663669287221368</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>0.8516363705588597</v>
+        <v>0.9807851014692465</v>
       </c>
       <c r="B83" t="n">
-        <v>0.9164942114467742</v>
+        <v>0.7333657148596476</v>
       </c>
       <c r="C83" t="n">
-        <v>0.9940997320270676</v>
+        <v>0.4976063521453536</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>0.578618223652045</v>
+        <v>0.7609522903011572</v>
       </c>
       <c r="B84" t="n">
-        <v>0.4179536733685759</v>
+        <v>0.5168750603939039</v>
       </c>
       <c r="C84" t="n">
-        <v>0.7283774774850734</v>
+        <v>0.1274035338864198</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>0.07146350781043842</v>
+        <v>0.7061203930491224</v>
       </c>
       <c r="B85" t="n">
-        <v>0.7538178944472897</v>
+        <v>0.6890543270543302</v>
       </c>
       <c r="C85" t="n">
-        <v>0.4353957080558639</v>
+        <v>0.1304580948890735</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>0.9350234525379962</v>
+        <v>0.721311809645875</v>
       </c>
       <c r="B86" t="n">
-        <v>0.2029686241321239</v>
+        <v>0.5450958930623314</v>
       </c>
       <c r="C86" t="n">
-        <v>0.9453079146861429</v>
+        <v>0.02709235561694801</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>0.3941496602074946</v>
+        <v>0.6228586294910202</v>
       </c>
       <c r="B87" t="n">
-        <v>0.9306411172826856</v>
+        <v>0.5491129259266241</v>
       </c>
       <c r="C87" t="n">
-        <v>0.1799248044267657</v>
+        <v>0.2155836423593378</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>0.7157188250942534</v>
+        <v>0.3481321490411865</v>
       </c>
       <c r="B88" t="n">
-        <v>0.3542437345992165</v>
+        <v>0.8521986590370128</v>
       </c>
       <c r="C88" t="n">
-        <v>0.8552053170642878</v>
+        <v>0.04264210435144045</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>0.05212695734308359</v>
+        <v>0.4975113851099219</v>
       </c>
       <c r="B89" t="n">
-        <v>0.5618055880113517</v>
+        <v>0.4126136315767233</v>
       </c>
       <c r="C89" t="n">
-        <v>0.0603421569177508</v>
+        <v>0.03607906069028866</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>0.2369466851270258</v>
+        <v>0.9721339832940058</v>
       </c>
       <c r="B90" t="n">
-        <v>0.4155398900534286</v>
+        <v>0.5991480326177639</v>
       </c>
       <c r="C90" t="n">
-        <v>0.7159862303151486</v>
+        <v>0.5170400306905084</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>0.4645734127804664</v>
+        <v>0.1587050192313649</v>
       </c>
       <c r="B91" t="n">
-        <v>0.2250908996478669</v>
+        <v>0.2912952634189143</v>
       </c>
       <c r="C91" t="n">
-        <v>0.8773191864458413</v>
+        <v>0.7410801506625332</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0.3965856510387251</v>
+        <v>0.3239604522420469</v>
       </c>
       <c r="B92" t="n">
-        <v>0.2770626591620254</v>
+        <v>0.8475767908780542</v>
       </c>
       <c r="C92" t="n">
-        <v>0.8763600240689823</v>
+        <v>0.4951961073647936</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>0.540405212040195</v>
+        <v>0.7364813775447006</v>
       </c>
       <c r="B93" t="n">
-        <v>0.379165250233039</v>
+        <v>0.2988296837242103</v>
       </c>
       <c r="C93" t="n">
-        <v>0.8745527654242466</v>
+        <v>0.4547839106545932</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>0.9416386881017255</v>
+        <v>0.6408210807652978</v>
       </c>
       <c r="B94" t="n">
-        <v>0.1679685085570363</v>
+        <v>0.01649383075234567</v>
       </c>
       <c r="C94" t="n">
-        <v>0.3716302140785965</v>
+        <v>0.08241983486212801</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>0.5020026259790688</v>
+        <v>0.4019958180643662</v>
       </c>
       <c r="B95" t="n">
-        <v>0.8348990767311817</v>
+        <v>0.4870849834415115</v>
       </c>
       <c r="C95" t="n">
-        <v>0.865982663413316</v>
+        <v>0.6101938718512822</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>0.3666016662544316</v>
+        <v>0.3264578098048514</v>
       </c>
       <c r="B96" t="n">
-        <v>0.1474795027860196</v>
+        <v>0.6695938794265895</v>
       </c>
       <c r="C96" t="n">
-        <v>0.8288396867948219</v>
+        <v>0.4061459811709425</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>0.2269651200852236</v>
+        <v>0.59947169502835</v>
       </c>
       <c r="B97" t="n">
-        <v>0.2516599687949611</v>
+        <v>0.1990156706955766</v>
       </c>
       <c r="C97" t="n">
-        <v>0.3108526510245896</v>
+        <v>0.3034220716905115</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>0.6586540905034437</v>
+        <v>0.2194676102387576</v>
       </c>
       <c r="B98" t="n">
-        <v>0.7708474677142754</v>
+        <v>0.6848122271828919</v>
       </c>
       <c r="C98" t="n">
-        <v>0.4197523026144331</v>
+        <v>0.3704702515758516</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>0.8566340214548899</v>
+        <v>0.3401102663773643</v>
       </c>
       <c r="B99" t="n">
-        <v>0.5542881314698378</v>
+        <v>0.480644452263608</v>
       </c>
       <c r="C99" t="n">
-        <v>0.7537607364185965</v>
+        <v>0.7692431511733557</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>0.05870420473629145</v>
+        <v>0.8929218316564272</v>
       </c>
       <c r="B100" t="n">
-        <v>0.988645517212568</v>
+        <v>0.3768718710811465</v>
       </c>
       <c r="C100" t="n">
-        <v>0.5062514734827349</v>
+        <v>0.5878196875070112</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>0.1439141791287202</v>
+        <v>0.5811365882406228</v>
       </c>
       <c r="B101" t="n">
-        <v>0.4650613920021659</v>
+        <v>0.7700890405502169</v>
       </c>
       <c r="C101" t="n">
-        <v>0.5872963238083758</v>
+        <v>0.4179238099094005</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fecha y hora inicio</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Isc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-03 10:00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>